<commit_message>
docs(tc): 09-04~06 분을 TC 에 등재한다 — 143 → 174행
정산 두 단계 · 하이패스 · 자동 배정 · 「이동」 이 TC 에 «한 줄도 없었다».
TC 생성기가 생긴 것이 09-08 이라 그 전에 확인한 것이 옮겨지지 않았고,
검증 결과 문서 12.6.17~20 이 유일한 기록이었다.

- 적합 28행 등재 (정산 두 단계 7 · 하이패스 읽기/붙이기 5 · 대조/대납 4 ·
  자동 배정/고치기 7 · 「이동」과 길찾기 5)
- 미수행 3행 (실적 창 하이패스 «고르기 화면» · 건별 하이패스 메일 ·
  네이버 링크가 실제로 열리는지) — 적합으로 «바꾸지 않고» 노란 칸으로 내렸다

🔑 값은 한 줄도 지어내지 않았다. 전부 «그날 커밋 본문의 「■ 검증 / ■ 실측」 블록»
   에서 옮겼다 — 커밋 메시지가 검증 기록의 정본 노릇을 한다.
⚠ 기능을 넣는 «그 턴에» 이 파일도 함께 고칠 것. 미루면 근거를 다시 캐야 한다.

확인 — 내려받은 첨부가 174행이고 로컬과 SHA256 이 같다.
적합인데 확인자 빈 행 0 · 미수행인데 확인자 채워진 행 0 · 확인 날짜는 전부 비움.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/testcase/TC_업무_현황_대시보드.xlsx
+++ b/docs/testcase/TC_업무_현황_대시보드.xlsx
@@ -756,7 +756,7 @@
     <row r="15" ht="24" customHeight="1">
       <c r="A15" s="7" t="inlineStr">
         <is>
-          <t>적합 137건 · 미수행 6건 · 부적합 0건</t>
+          <t>적합 165건 · 미수행 9건 · 부적합 0건</t>
         </is>
       </c>
       <c r="B15" s="5" t="n"/>
@@ -789,7 +789,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I146"/>
+  <dimension ref="A1:I177"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -5403,17 +5403,17 @@
       </c>
       <c r="B109" s="10" t="inlineStr">
         <is>
-          <t>휴가</t>
+          <t>정산</t>
         </is>
       </c>
       <c r="C109" s="4" t="inlineStr">
         <is>
-          <t>지난 날짜에 넣으면 신청 메일이 «안» 가는가?</t>
+          <t>사람별로 확정하면 «그 사람» 실적만 잠기는가?</t>
         </is>
       </c>
       <c r="D109" s="4" t="inlineStr">
         <is>
-          <t>지난 날짜로 휴가를 넣고 서버 발송 기록 확인</t>
+          <t>한 사람만 확정한 뒤 나머지 사람의 실적이 열려 있는지 확인</t>
         </is>
       </c>
       <c r="E109" s="11" t="inlineStr">
@@ -5429,12 +5429,12 @@
       <c r="G109" s="10" t="inlineStr"/>
       <c r="H109" s="4" t="inlineStr">
         <is>
-          <t>나가면 plan_date 와 오늘을 맞대는 판정 확인</t>
+          <t>전원이 잠기면 잠금 UPDATE 에 worker_id 조건이 있는지 확인</t>
         </is>
       </c>
       <c r="I109" s="4" t="inlineStr">
         <is>
-          <t>로그 skip(backfill) — 9/07·9/05 넷(신청·취소) 다 안 감</t>
+          <t>이건호 21/21 잠김 · 나머지 4명 25건은 열림 (종전이면 46건 전부 잠겼다)</t>
         </is>
       </c>
     </row>
@@ -5446,17 +5446,17 @@
       </c>
       <c r="B110" s="12" t="inlineStr">
         <is>
-          <t>휴가</t>
+          <t>정산</t>
         </is>
       </c>
       <c r="C110" s="13" t="inlineStr">
         <is>
-          <t>오늘·앞날은 «그대로» 신청 메일이 가는가?</t>
+          <t>한 명만 확정돼도 「정산 완료」로 보이지 않는가?</t>
         </is>
       </c>
       <c r="D110" s="13" t="inlineStr">
         <is>
-          <t>오늘·앞날로 넣고 서버 발송 기록 확인</t>
+          <t>한 사람만 확정한 뒤 상단 배지 확인</t>
         </is>
       </c>
       <c r="E110" s="14" t="inlineStr">
@@ -5472,12 +5472,12 @@
       <c r="G110" s="12" t="inlineStr"/>
       <c r="H110" s="13" t="inlineStr">
         <is>
-          <t>안 가면 판정이 지나치게 넓은지 확인</t>
+          <t>완료로 보이면 배지 계산을 확인</t>
         </is>
       </c>
       <c r="I110" s="13" t="inlineStr">
         <is>
-          <t>9/10·9/13 신청·취소 넷 다 나감 — 막아 버리면 안 된다</t>
+          <t>「1/5명 정산 완료」</t>
         </is>
       </c>
     </row>
@@ -5489,17 +5489,17 @@
       </c>
       <c r="B111" s="10" t="inlineStr">
         <is>
-          <t>휴가</t>
+          <t>정산</t>
         </is>
       </c>
       <c r="C111" s="4" t="inlineStr">
         <is>
-          <t>지난 날짜가 «승인 대기»에 쌓이지 않는가?</t>
+          <t>확정 뒤 값이 달라지면 확정액과 현재액을 «둘 다» 보이는가?</t>
         </is>
       </c>
       <c r="D111" s="4" t="inlineStr">
         <is>
-          <t>승인권자 계정으로 대기 목록을 넣기 전후로 세어 본다</t>
+          <t>확정 후 단가를 바꾸고 줄과 합계 확인</t>
         </is>
       </c>
       <c r="E111" s="11" t="inlineStr">
@@ -5515,12 +5515,12 @@
       <c r="G111" s="10" t="inlineStr"/>
       <c r="H111" s="4" t="inlineStr">
         <is>
-          <t>늘어나면 자동 승인이 안 걸린 것</t>
+          <t>한쪽만 보이면 확정 금액을 싣는지 확인</t>
         </is>
       </c>
       <c r="I111" s="4" t="inlineStr">
         <is>
-          <t>넣기 전 0 → 지난 날짜 2건 넣은 뒤에도 0</t>
+          <t>단가 100→150 → 「30,000원 → 현재 45,000원」 · 합계는 확정 금액 30,000원 유지</t>
         </is>
       </c>
     </row>
@@ -5532,17 +5532,17 @@
       </c>
       <c r="B112" s="12" t="inlineStr">
         <is>
-          <t>휴가</t>
+          <t>정산</t>
         </is>
       </c>
       <c r="C112" s="13" t="inlineStr">
         <is>
-          <t>자동 승인된 것을 «사람이 승인한 것»과 구분할 수 있는가?</t>
+          <t>1차 안내가 나가면 그 사람 실적이 잠기는가?</t>
         </is>
       </c>
       <c r="D112" s="13" t="inlineStr">
         <is>
-          <t>저장된 approval 과 approved_by_id 확인</t>
+          <t>1차 안내를 보내고 상태·잠금 건수·발송 기록 확인</t>
         </is>
       </c>
       <c r="E112" s="14" t="inlineStr">
@@ -5558,12 +5558,12 @@
       <c r="G112" s="12" t="inlineStr"/>
       <c r="H112" s="13" t="inlineStr">
         <is>
-          <t>승인자가 채워지면 「누가 승인했다」가 거짓이 된다</t>
+          <t>안 잠기면 안내와 잠금이 한 흐름인지 확인</t>
         </is>
       </c>
       <c r="I112" s="13" t="inlineStr">
         <is>
-          <t>approved + approved_by_id = null · 승인 시각은 찍힌다</t>
+          <t>notified · 21/21 잠금 · 메일 실제 발송(ok:true)</t>
         </is>
       </c>
     </row>
@@ -5575,17 +5575,17 @@
       </c>
       <c r="B113" s="10" t="inlineStr">
         <is>
-          <t>휴가</t>
+          <t>정산</t>
         </is>
       </c>
       <c r="C113" s="4" t="inlineStr">
         <is>
-          <t>지난 날짜를 지울 때도 취소 메일이 «안» 가는가?</t>
+          <t>입금할 것이 없는 사람은 메일 없이 완료로 가는가?</t>
         </is>
       </c>
       <c r="D113" s="4" t="inlineStr">
         <is>
-          <t>지난 날짜 건을 지우고 발송 기록 확인</t>
+          <t>0원인 사람에게 1차 안내를 돌려 상태와 발송 기록 확인</t>
         </is>
       </c>
       <c r="E113" s="11" t="inlineStr">
@@ -5601,12 +5601,12 @@
       <c r="G113" s="10" t="inlineStr"/>
       <c r="H113" s="4" t="inlineStr">
         <is>
-          <t>가면 취소 경로에도 같은 판정이 걸렸는지 확인</t>
+          <t>메일이 가면 0원 판정을 확인</t>
         </is>
       </c>
       <c r="I113" s="4" t="inlineStr">
         <is>
-          <t>신청이 안 갔는데 취소만 가면 «없던 신청»이 취소된 것으로 읽힌다</t>
+          <t>김동현·송지형은 그 자리에서 settled · 송지형 때 메일은 나가지 않았다</t>
         </is>
       </c>
     </row>
@@ -5618,17 +5618,17 @@
       </c>
       <c r="B114" s="12" t="inlineStr">
         <is>
-          <t>휴가</t>
+          <t>정산</t>
         </is>
       </c>
       <c r="C114" s="13" t="inlineStr">
         <is>
-          <t>날짜가 섞였을 때 화면이 «갈라서» 묻는가?</t>
+          <t>잠긴 뒤 수정과 완료 뒤 수정이 갈라지는가?</t>
         </is>
       </c>
       <c r="D114" s="13" t="inlineStr">
         <is>
-          <t>지난 날짜와 오늘을 함께 골라 확인 창 문구를 읽는다</t>
+          <t>notified 와 settled 각각에서 승인권자 PATCH 시도</t>
         </is>
       </c>
       <c r="E114" s="14" t="inlineStr">
@@ -5644,12 +5644,12 @@
       <c r="G114" s="12" t="inlineStr"/>
       <c r="H114" s="13" t="inlineStr">
         <is>
-          <t>한 줄로 뭉뚱그리면 어느 쪽이 갔는지 알 수 없다</t>
+          <t>둘 다 통과하면 상태별 잠금 조건 확인</t>
         </is>
       </c>
       <c r="I114" s="13" t="inlineStr">
         <is>
-          <t>「지난 1건은 정리 기록…나머지 1건만 신청 메일」 · 전부 지난 날짜면 「넣을까요?」</t>
+          <t>notified → 200 / settled → 409</t>
         </is>
       </c>
     </row>
@@ -5661,17 +5661,17 @@
       </c>
       <c r="B115" s="10" t="inlineStr">
         <is>
-          <t>휴가</t>
+          <t>정산</t>
         </is>
       </c>
       <c r="C115" s="4" t="inlineStr">
         <is>
-          <t>시각을 고르면 시스템이 시간을 세는가?</t>
+          <t>2차 입금 확인으로 완료되는가?</t>
         </is>
       </c>
       <c r="D115" s="4" t="inlineStr">
         <is>
-          <t>종일·09:00~18:00·09:00~13:00 등 여덟 가지로 등록해 값 확인</t>
+          <t>complete 를 부르고 상태 확인 · 대기가 없는데 또 불러 본다</t>
         </is>
       </c>
       <c r="E115" s="11" t="inlineStr">
@@ -5687,12 +5687,12 @@
       <c r="G115" s="10" t="inlineStr"/>
       <c r="H115" s="4" t="inlineStr">
         <is>
-          <t>값이 다르면 근무·점심 시각 상수와 겹침 계산 확인</t>
+          <t>완료가 안 되면 2차 경로 확인</t>
         </is>
       </c>
       <c r="I115" s="4" t="inlineStr">
         <is>
-          <t>8/8 일치 — 종일 8 · 09~18 8 · 09~13 3 · 13~18 5 · 11~14 2 · 끝이 앞서면 0</t>
+          <t>settled · 대기 없으면 404 안내</t>
         </is>
       </c>
     </row>
@@ -5704,17 +5704,17 @@
       </c>
       <c r="B116" s="12" t="inlineStr">
         <is>
-          <t>휴가</t>
+          <t>하이패스</t>
         </is>
       </c>
       <c r="C116" s="13" t="inlineStr">
         <is>
-          <t>점심시간이 휴가에서 빠지는가?</t>
+          <t>명세 엑셀을 제대로 읽는가?</t>
         </is>
       </c>
       <c r="D116" s="13" t="inlineStr">
         <is>
-          <t>09:00~13:00 으로 등록해 3시간인지 확인</t>
+          <t>실물 명세 파일을 올려 건수·합계를 파일 머리말과 대조</t>
         </is>
       </c>
       <c r="E116" s="14" t="inlineStr">
@@ -5730,12 +5730,12 @@
       <c r="G116" s="12" t="inlineStr"/>
       <c r="H116" s="13" t="inlineStr">
         <is>
-          <t>4시간이면 점심 구간과의 겹침을 빼는지 확인</t>
+          <t>다르면 파싱 규칙을 확인</t>
         </is>
       </c>
       <c r="I116" s="13" t="inlineStr">
         <is>
-          <t>3시간 — 점심 전까지(09~12)도 3시간이라 겹칠 때만 빠진다</t>
+          <t>66건 · 212,640원 — 파일 머리말(전체건수 66 · 212,640)과 일치</t>
         </is>
       </c>
     </row>
@@ -5747,17 +5747,17 @@
       </c>
       <c r="B117" s="10" t="inlineStr">
         <is>
-          <t>휴가</t>
+          <t>하이패스</t>
         </is>
       </c>
       <c r="C117" s="4" t="inlineStr">
         <is>
-          <t>「반차」 단추가 사라지고 시각 고르개가 나오는가?</t>
+          <t>카드번호로 차량을 찾고 그 카드를 기억하는가?</t>
         </is>
       </c>
       <c r="D117" s="4" t="inlineStr">
         <is>
-          <t>운영 화면에서 휴가 유형을 골라 단추 목록 확인</t>
+          <t>카드 미등록 상태로 올린 뒤 차량을 골라 다시 올린다</t>
         </is>
       </c>
       <c r="E117" s="11" t="inlineStr">
@@ -5773,12 +5773,12 @@
       <c r="G117" s="10" t="inlineStr"/>
       <c r="H117" s="4" t="inlineStr">
         <is>
-          <t>반차가 남아 있으면 배포본이 옛것인지 확인</t>
+          <t>매번 물으면 카드를 차량에 기억시키는지 확인</t>
         </is>
       </c>
       <c r="I117" s="4" t="inlineStr">
         <is>
-          <t>종류 연차·병가·포상·공가·기타 / 길이 종일(8시간)·시간 지정</t>
+          <t>미등록이면 404 need_vehicle · 한 번 고르면 다음부터 묻지 않는다</t>
         </is>
       </c>
     </row>
@@ -5790,17 +5790,17 @@
       </c>
       <c r="B118" s="12" t="inlineStr">
         <is>
-          <t>휴가</t>
+          <t>하이패스</t>
         </is>
       </c>
       <c r="C118" s="13" t="inlineStr">
         <is>
-          <t>지난 휴가가 종일 8시간·반차 4시간으로 환산됐는가?</t>
+          <t>같은 파일을 두 번 올려도 겹쳐 들어가지 않는가?</t>
         </is>
       </c>
       <c r="D118" s="13" t="inlineStr">
         <is>
-          <t>운영 DB 에 마이그레이션 035 적용 후 환산 결과 확인</t>
+          <t>같은 파일을 재업로드해 결과 수 확인</t>
         </is>
       </c>
       <c r="E118" s="14" t="inlineStr">
@@ -5816,12 +5816,12 @@
       <c r="G118" s="12" t="inlineStr"/>
       <c r="H118" s="13" t="inlineStr">
         <is>
-          <t>빈 값이 남으면 UPDATE 조건 확인</t>
+          <t>늘어나면 겹침 인덱스를 확인</t>
         </is>
       </c>
       <c r="I118" s="13" t="inlineStr">
         <is>
-          <t>운영 5건 모두 종일 → 8시간 · 시간 없는 휴가 0건</t>
+          <t>inserted 0 · duplicated 66 — 「이미 있던 것」을 숨기지 않고 함께 보여 준다</t>
         </is>
       </c>
     </row>
@@ -5833,17 +5833,17 @@
       </c>
       <c r="B119" s="10" t="inlineStr">
         <is>
-          <t>휴가</t>
+          <t>하이패스</t>
         </is>
       </c>
       <c r="C119" s="4" t="inlineStr">
         <is>
-          <t>연차 집계가 «일과 시간» 을 함께 내는가?</t>
+          <t>통행 날짜가 하루 밀리지 않는가?</t>
         </is>
       </c>
       <c r="D119" s="4" t="inlineStr">
         <is>
-          <t>연차 요약에서 부여·사용·잔여 값 확인</t>
+          <t>월초 구간으로 조회해 마지막 줄의 날짜 확인</t>
         </is>
       </c>
       <c r="E119" s="11" t="inlineStr">
@@ -5859,12 +5859,12 @@
       <c r="G119" s="10" t="inlineStr"/>
       <c r="H119" s="4" t="inlineStr">
         <is>
-          <t>한쪽만 나오면 집계 응답에 시간 칸이 있는지 확인</t>
+          <t>하루 이르면 UTC 로 읽고 있는지 확인</t>
         </is>
       </c>
       <c r="I119" s="4" t="inlineStr">
         <is>
-          <t>부여 21일/168시간 · 하루 8시간 · 잔여도 양쪽 표시</t>
+          <t>9/1~9/4 조회에 마지막 줄이 09-04 (UTC 였다면 09-03)</t>
         </is>
       </c>
     </row>
@@ -5876,17 +5876,17 @@
       </c>
       <c r="B120" s="12" t="inlineStr">
         <is>
-          <t>휴가</t>
+          <t>하이패스</t>
         </is>
       </c>
       <c r="C120" s="13" t="inlineStr">
         <is>
-          <t>「공가」를 종류로 고를 수 있고 사유를 적을 수 있는가?</t>
+          <t>통행을 붙이고 떼면 실적 금액이 따라오는가?</t>
         </is>
       </c>
       <c r="D120" s="13" t="inlineStr">
         <is>
-          <t>운영 화면에서 공가를 고르고 사유 칸 확인</t>
+          <t>API 로 3건 붙이고 1건 떼며 실적의 통행료 확인</t>
         </is>
       </c>
       <c r="E120" s="14" t="inlineStr">
@@ -5902,12 +5902,12 @@
       <c r="G120" s="12" t="inlineStr"/>
       <c r="H120" s="13" t="inlineStr">
         <is>
-          <t>안 보이면 마이그레이션 033 이 운영 DB 에 들어갔는지 확인</t>
+          <t>안 따라오면 합산 경로를 확인</t>
         </is>
       </c>
       <c r="I120" s="13" t="inlineStr">
         <is>
-          <t>종류 다섯에 공가 확인(운영 화면) · 사유 칸은 같은 판 화면에서 확인 · 예비군·경조용</t>
+          <t>2,500 → 4,300 → 6,600 · 1건 떼니 4,800</t>
         </is>
       </c>
     </row>
@@ -5919,17 +5919,17 @@
       </c>
       <c r="B121" s="10" t="inlineStr">
         <is>
-          <t>회의록</t>
+          <t>하이패스</t>
         </is>
       </c>
       <c r="C121" s="4" t="inlineStr">
         <is>
-          <t>작성자를 직원 목록에서 고르거나 직접 적을 수 있는가?</t>
+          <t>통행마다 「그날 그 차를 쓴 실적」을 맞대 방향을 붙이는가?</t>
         </is>
       </c>
       <c r="D121" s="4" t="inlineStr">
         <is>
-          <t>회의록을 만들며 두 가지 방식으로 저장한 뒤 다시 조회</t>
+          <t>입금·환급·「골라야 함」 세 갈래를 임시 실적·통행으로 만들어 확인</t>
         </is>
       </c>
       <c r="E121" s="11" t="inlineStr">
@@ -5945,12 +5945,12 @@
       <c r="G121" s="10" t="inlineStr"/>
       <c r="H121" s="4" t="inlineStr">
         <is>
-          <t>한쪽만 남으면 «둘 중 하나만» 담는 조건 확인</t>
+          <t>값이 다르면 대조 조건(날짜·차량)을 확인</t>
         </is>
       </c>
       <c r="I121" s="4" t="inlineStr">
         <is>
-          <t>직접 입력 → 글자로 · 목록 선택 → 번호로. 양쪽에 동시에 남지 않는다</t>
+          <t>세 갈래 모두 제 값 · 지운 뒤 원래 43건(회사 부담 26 · 해당 없음 17)으로 복원</t>
         </is>
       </c>
     </row>
@@ -5962,17 +5962,17 @@
       </c>
       <c r="B122" s="12" t="inlineStr">
         <is>
-          <t>회의록</t>
+          <t>하이패스</t>
         </is>
       </c>
       <c r="C122" s="13" t="inlineStr">
         <is>
-          <t>회의 내용에 서식(굵게·크기·색)을 넣을 수 있는가?</t>
+          <t>개인카드로 낸 통행료를 주 사용자에게 지급하는가?</t>
         </is>
       </c>
       <c r="D122" s="13" t="inlineStr">
         <is>
-          <t>글을 골라 B·크게·빨강을 눌러 실제 저장값 확인</t>
+          <t>개인카드 차량의 «붙은» 통행 합계와 대납 금액을 대조</t>
         </is>
       </c>
       <c r="E122" s="14" t="inlineStr">
@@ -5988,12 +5988,12 @@
       <c r="G122" s="12" t="inlineStr"/>
       <c r="H122" s="13" t="inlineStr">
         <is>
-          <t>안 걸리면 고른 글이 풀렸는지(마우스 누름 차단) 확인</t>
+          <t>다르면 붙은 것만 세는지 확인</t>
         </is>
       </c>
       <c r="I122" s="13" t="inlineStr">
         <is>
-          <t>font-weight·font-size·color 가 걸리고 저장 후에도 남는다</t>
+          <t>이건호 대납 5,600원 = 붙은 통행 4건 × 1,400 과 일치</t>
         </is>
       </c>
     </row>
@@ -6005,17 +6005,17 @@
       </c>
       <c r="B123" s="10" t="inlineStr">
         <is>
-          <t>회의록</t>
+          <t>하이패스</t>
         </is>
       </c>
       <c r="C123" s="4" t="inlineStr">
         <is>
-          <t>붙여 넣은 글이 «글자만» 들어오는가?</t>
+          <t>대납과 청구 두 갈래가 «함께» 잡히는가?</t>
         </is>
       </c>
       <c r="D123" s="4" t="inlineStr">
         <is>
-          <t>배경색·글꼴이 든 글을 편집기에 붙여 넣고 들어간 값 확인</t>
+          <t>남이 그 차를 개인 사용한 임시 실적을 넣어 양쪽 금액 확인</t>
         </is>
       </c>
       <c r="E123" s="11" t="inlineStr">
@@ -6031,12 +6031,12 @@
       <c r="G123" s="10" t="inlineStr"/>
       <c r="H123" s="4" t="inlineStr">
         <is>
-          <t>배경색이 따라오면 붙여 넣기 가로채기 확인</t>
+          <t>한쪽만 잡히면 정산 계산에 두 갈래가 다 얹혔는지 확인</t>
         </is>
       </c>
       <c r="I123" s="4" t="inlineStr">
         <is>
-          <t>글자만 들어감 — background·font-family 안 따라옴 · 흰 바탕에 흰 글씨를 막는다</t>
+          <t>김동현 청구 1,440 · 이건호 대납 7,040 · 되돌리니 원복</t>
         </is>
       </c>
     </row>
@@ -6048,17 +6048,17 @@
       </c>
       <c r="B124" s="12" t="inlineStr">
         <is>
-          <t>회의록</t>
+          <t>하이패스</t>
         </is>
       </c>
       <c r="C124" s="13" t="inlineStr">
         <is>
-          <t>옛 회의록(서식 없는 글)이 그대로 보이는가?</t>
+          <t>주 사용자가 없는 차는 「개인카드」를 켤 수 없는가?</t>
         </is>
       </c>
       <c r="D124" s="13" t="inlineStr">
         <is>
-          <t>서식 없이 적힌 회의록을 열어 줄바꿈·본문 확인</t>
+          <t>주 사용자 없는 차의 체크칸 확인</t>
         </is>
       </c>
       <c r="E124" s="14" t="inlineStr">
@@ -6074,12 +6074,12 @@
       <c r="G124" s="12" t="inlineStr"/>
       <c r="H124" s="13" t="inlineStr">
         <is>
-          <t>뭉개지면 글자를 서식으로 바꾸는 경로 확인</t>
+          <t>켜지면 화면·서버·DB CHECK 셋 중 어디가 빠졌는지 확인</t>
         </is>
       </c>
       <c r="I124" s="13" t="inlineStr">
         <is>
-          <t>줄바꿈 유지 — 운영의 지난 주간회의로 확인</t>
+          <t>회색으로 잠겨 있다 — 줄 사람이 없으면 그 돈은 갈 곳을 잃는다</t>
         </is>
       </c>
     </row>
@@ -6091,17 +6091,17 @@
       </c>
       <c r="B125" s="10" t="inlineStr">
         <is>
-          <t>회의록</t>
+          <t>하이패스</t>
         </is>
       </c>
       <c r="C125" s="4" t="inlineStr">
         <is>
-          <t>위험한 글이 «보는 화면» 에서 걸러지는가?</t>
+          <t>후보가 «정확히 하나» 일 때만 자동으로 붙는가?</t>
         </is>
       </c>
       <c r="D125" s="4" t="inlineStr">
         <is>
-          <t>DB 에 직접 심고 회의록을 열어 실행 여부 확인</t>
+          <t>올린 뒤 자동 배정 결과 확인</t>
         </is>
       </c>
       <c r="E125" s="11" t="inlineStr">
@@ -6117,12 +6117,12 @@
       <c r="G125" s="10" t="inlineStr"/>
       <c r="H125" s="4" t="inlineStr">
         <is>
-          <t>실행되면 그리기 직전의 거르개 확인</t>
+          <t>둘 이상인데 붙으면 후보 수 판정을 확인</t>
         </is>
       </c>
       <c r="I125" s="4" t="inlineStr">
         <is>
-          <t>script·img·iframe 0개 · javascript: 주소 떨어짐 · 색·목록 서식은 남음</t>
+          <t>1건 붙음 · 애매 0 · 실적 없는 3건은 사람에게 남김</t>
         </is>
       </c>
     </row>
@@ -6134,17 +6134,17 @@
       </c>
       <c r="B126" s="12" t="inlineStr">
         <is>
-          <t>회의록</t>
+          <t>하이패스</t>
         </is>
       </c>
       <c r="C126" s="13" t="inlineStr">
         <is>
-          <t>위험한 글이 «고치는 화면» 에서도 걸러지는가?</t>
+          <t>「정산 제외」가 기록을 남기고 금액에서만 빼는가?</t>
         </is>
       </c>
       <c r="D126" s="13" t="inlineStr">
         <is>
-          <t>같은 글로 [내용 수정] 을 눌러 실행 여부 확인</t>
+          <t>제외한 뒤 금액과 목록을 확인하고 풀어서 되돌린다</t>
         </is>
       </c>
       <c r="E126" s="14" t="inlineStr">
@@ -6160,12 +6160,12 @@
       <c r="G126" s="12" t="inlineStr"/>
       <c r="H126" s="13" t="inlineStr">
         <is>
-          <t>실행되면 편집기에 담을 때도 거르는지 확인</t>
+          <t>줄이 사라지면 지우기로 구현된 것</t>
         </is>
       </c>
       <c r="I126" s="13" t="inlineStr">
         <is>
-          <t>🔴 처음 판은 여기서 &lt;img onerror&gt; 가 터졌다 — 고친 뒤 재확인</t>
+          <t>4,440 → 3,000 · 풀면 완전 복원 · 「누구 것이었나」는 남는다</t>
         </is>
       </c>
     </row>
@@ -6177,17 +6177,17 @@
       </c>
       <c r="B127" s="10" t="inlineStr">
         <is>
-          <t>회의록</t>
+          <t>하이패스</t>
         </is>
       </c>
       <c r="C127" s="4" t="inlineStr">
         <is>
-          <t>발표 내용을 «본인 칸만» 고칠 수 있는가?</t>
+          <t>다른 직원에게 넘기면 방향대로 잡히는가?</t>
         </is>
       </c>
       <c r="D127" s="4" t="inlineStr">
         <is>
-          <t>다른 사람 번호로 저장 요청</t>
+          <t>환급·입금 두 방향으로 넘겨 금액을 확인한 뒤 되돌린다</t>
         </is>
       </c>
       <c r="E127" s="11" t="inlineStr">
@@ -6203,12 +6203,12 @@
       <c r="G127" s="10" t="inlineStr"/>
       <c r="H127" s="4" t="inlineStr">
         <is>
-          <t>저장되면 주소의 번호와 세션을 맞대는지 확인</t>
+          <t>방향이 없으면 billed_kind 를 받는지 확인</t>
         </is>
       </c>
       <c r="I127" s="4" t="inlineStr">
         <is>
-          <t>403 「본인의 발표 내용만 적을 수 있습니다」</t>
+          <t>환급 → 자차하이패스 1,440 / 입금 → 청구 1,440 · 되돌리면 원래대로</t>
         </is>
       </c>
     </row>
@@ -6220,17 +6220,17 @@
       </c>
       <c r="B128" s="12" t="inlineStr">
         <is>
-          <t>회의록</t>
+          <t>하이패스</t>
         </is>
       </c>
       <c r="C128" s="13" t="inlineStr">
         <is>
-          <t>관리자는 남의 발표 내용을 대신 넣을 수 있는가?</t>
+          <t>확정·제외한 건을 다시 손대지 못하게 막는가?</t>
         </is>
       </c>
       <c r="D128" s="13" t="inlineStr">
         <is>
-          <t>관리자 계정으로 다른 사람 칸에 저장</t>
+          <t>제외한 것 확정 · 확정한 것 넘기기·떼기를 각각 시도</t>
         </is>
       </c>
       <c r="E128" s="14" t="inlineStr">
@@ -6246,12 +6246,12 @@
       <c r="G128" s="12" t="inlineStr"/>
       <c r="H128" s="13" t="inlineStr">
         <is>
-          <t>막히면 등급 판정 확인</t>
+          <t>통과하면 알린 금액과 근거가 어긋난다</t>
         </is>
       </c>
       <c r="I128" s="13" t="inlineStr">
         <is>
-          <t>200 — 대리 입력은 허용한다</t>
+          <t>전부 409</t>
         </is>
       </c>
     </row>
@@ -6263,17 +6263,17 @@
       </c>
       <c r="B129" s="10" t="inlineStr">
         <is>
-          <t>회의록</t>
+          <t>하이패스</t>
         </is>
       </c>
       <c r="C129" s="4" t="inlineStr">
         <is>
-          <t>한 사람이 프로젝트마다 나눠 적을 수 있는가?</t>
+          <t>반려가 실적에서 떼지 않고 «제외»로 가는가?</t>
         </is>
       </c>
       <c r="D129" s="4" t="inlineStr">
         <is>
-          <t>같은 사람으로 프로젝트 둘 + 미지정 하나를 저장해 줄 수 확인</t>
+          <t>반려한 뒤 실적 번호와 상태 확인</t>
         </is>
       </c>
       <c r="E129" s="11" t="inlineStr">
@@ -6289,12 +6289,12 @@
       <c r="G129" s="10" t="inlineStr"/>
       <c r="H129" s="4" t="inlineStr">
         <is>
-          <t>한 줄로 덮이면 열쇠에 프로젝트가 들어갔는지 확인</t>
+          <t>떼어지면 「누구 것이었나」가 사라진다</t>
         </is>
       </c>
       <c r="I129" s="4" t="inlineStr">
         <is>
-          <t>3줄 유지 — 열쇠는 «회의 × 사람 × 프로젝트»</t>
+          <t>실적 125 를 유지한 채 제외로만</t>
         </is>
       </c>
     </row>
@@ -6306,17 +6306,17 @@
       </c>
       <c r="B130" s="12" t="inlineStr">
         <is>
-          <t>회의록</t>
+          <t>하이패스</t>
         </is>
       </c>
       <c r="C130" s="13" t="inlineStr">
         <is>
-          <t>같은 사람·같은 프로젝트에 다시 적으면 덮어쓰는가?</t>
+          <t>방향 없는 청구가 DB 에서 막히는가?</t>
         </is>
       </c>
       <c r="D130" s="13" t="inlineStr">
         <is>
-          <t>같은 자리에 두 번 저장해 줄 수와 내용 확인</t>
+          <t>billed_kind 를 비운 채 청구를 걸어 본다</t>
         </is>
       </c>
       <c r="E130" s="14" t="inlineStr">
@@ -6332,12 +6332,12 @@
       <c r="G130" s="12" t="inlineStr"/>
       <c r="H130" s="13" t="inlineStr">
         <is>
-          <t>줄이 늘면 겹침 열쇠 확인</t>
+          <t>들어가면 CHECK 의 IN 이 NULL 을 못 막는 것</t>
         </is>
       </c>
       <c r="I130" s="13" t="inlineStr">
         <is>
-          <t>줄 수 그대로 · 내용만 바뀜</t>
+          <t>🔴 처음엔 «안 막았다» — NULL IN(…) 은 FALSE 가 아니라 NULL 이다. coalesce 로 고친 뒤 «막히는 것» 까지 확인</t>
         </is>
       </c>
     </row>
@@ -6349,17 +6349,17 @@
       </c>
       <c r="B131" s="10" t="inlineStr">
         <is>
-          <t>회의록</t>
+          <t>하이패스</t>
         </is>
       </c>
       <c r="C131" s="4" t="inlineStr">
         <is>
-          <t>프로젝트를 안 고른 줄이 여러 개로 쌓이지 않는가?</t>
+          <t>정정 요청에 사유를 요구하는가?</t>
         </is>
       </c>
       <c r="D131" s="4" t="inlineStr">
         <is>
-          <t>프로젝트 없이 두 번 저장해 줄 수 확인</t>
+          <t>사유 없이·사유 있이 각각 요청</t>
         </is>
       </c>
       <c r="E131" s="11" t="inlineStr">
@@ -6375,12 +6375,12 @@
       <c r="G131" s="10" t="inlineStr"/>
       <c r="H131" s="4" t="inlineStr">
         <is>
-          <t>두 줄이면 NULL 을 빈 글자로 바꿔 잠갔는지 확인</t>
+          <t>사유 없이 통과하면 근거가 남지 않는다</t>
         </is>
       </c>
       <c r="I131" s="4" t="inlineStr">
         <is>
-          <t>🔴 NULL 끼리는 서로 같지 않아 그냥 UNIQUE 로는 «안 막힌다» · 1줄 확인</t>
+          <t>없으면 400 · 있으면 200 · 확정 뒤에 답하면 409</t>
         </is>
       </c>
     </row>
@@ -6392,17 +6392,17 @@
       </c>
       <c r="B132" s="12" t="inlineStr">
         <is>
-          <t>회의록</t>
+          <t>일정</t>
         </is>
       </c>
       <c r="C132" s="13" t="inlineStr">
         <is>
-          <t>프로젝트를 옮기면 옛 줄이 남지 않는가?</t>
+          <t>장소 쌍 거리가 방향을 가리지 않는가?</t>
         </is>
       </c>
       <c r="D132" s="13" t="inlineStr">
         <is>
-          <t>적어 둔 줄의 프로젝트를 바꿔 저장한 뒤 목록 확인</t>
+          <t>한 방향으로 저장한 뒤 뒤집어 조회</t>
         </is>
       </c>
       <c r="E132" s="14" t="inlineStr">
@@ -6418,12 +6418,12 @@
       <c r="G132" s="12" t="inlineStr"/>
       <c r="H132" s="13" t="inlineStr">
         <is>
-          <t>두 자리에 남으면 옮길 때 옛 줄을 먼저 지우는지 확인</t>
+          <t>두 줄로 남으면 한쪽만 고쳐져 조용히 어긋난다</t>
         </is>
       </c>
       <c r="I132" s="13" t="inlineStr">
         <is>
-          <t>화면에서 확인 — 개수 3 그대로, 옛 프로젝트에서 사라짐</t>
+          <t>SKIPC↔삼양화학 87.4km/75분 — 뒤집어 조회해도 같은 줄</t>
         </is>
       </c>
     </row>
@@ -6435,17 +6435,17 @@
       </c>
       <c r="B133" s="10" t="inlineStr">
         <is>
-          <t>회의록</t>
+          <t>일정</t>
         </is>
       </c>
       <c r="C133" s="4" t="inlineStr">
         <is>
-          <t>적어 둔 것이 본문 아래에 «한 박스» 로 이어 붙는가?</t>
+          <t>유형에 안 맞는 방향·출발지를 서버가 지우는가?</t>
         </is>
       </c>
       <c r="D133" s="4" t="inlineStr">
         <is>
-          <t>회의록을 열어 본문과 발표 내용이 한 상자에 나오는지 확인</t>
+          <t>이동·왕복·출발로 각각 저장해 저장값 확인</t>
         </is>
       </c>
       <c r="E133" s="11" t="inlineStr">
@@ -6461,12 +6461,12 @@
       <c r="G133" s="10" t="inlineStr"/>
       <c r="H133" s="4" t="inlineStr">
         <is>
-          <t>따로 나오면 이어 붙이는 자리 확인</t>
+          <t>남으면 달력이 「A→B」라고 거짓말을 한다</t>
         </is>
       </c>
       <c r="I133" s="4" t="inlineStr">
         <is>
-          <t>🗣 이름과 📁 프로젝트가 함께 붙는다</t>
+          <t>이동 dir=이동·from=6·km=87.4 / 왕복·출발은 서버가 지움</t>
         </is>
       </c>
     </row>
@@ -6478,17 +6478,17 @@
       </c>
       <c r="B134" s="12" t="inlineStr">
         <is>
-          <t>회의록</t>
+          <t>일정</t>
         </is>
       </c>
       <c r="C134" s="13" t="inlineStr">
         <is>
-          <t>같은 글을 인원별·프로젝트별 두 가지로 묶어 볼 수 있는가?</t>
+          <t>「이동」이 달력에 출발지→도착지로 보이는가?</t>
         </is>
       </c>
       <c r="D134" s="13" t="inlineStr">
         <is>
-          <t>[🗣 인원별]/[📁 프로젝트별] 을 눌러 묶음이 뒤집히는지 확인</t>
+          <t>이동 일정을 등록해 달력 배지 확인</t>
         </is>
       </c>
       <c r="E134" s="14" t="inlineStr">
@@ -6504,12 +6504,12 @@
       <c r="G134" s="12" t="inlineStr"/>
       <c r="H134" s="13" t="inlineStr">
         <is>
-          <t>한쪽만 되면 묶는 기준만 바꾸는지 확인</t>
+          <t>한쪽만 나오면 배지 문구를 확인</t>
         </is>
       </c>
       <c r="I134" s="13" t="inlineStr">
         <is>
-          <t>인원별=사람→프로젝트 · 프로젝트별=프로젝트→사람 · 미지정은 늘 맨 뒤</t>
+          <t>「SKIPC→삼양화학 · QM6 · 편도」 / 출발은 「→삼양화학」</t>
         </is>
       </c>
     </row>
@@ -6521,17 +6521,17 @@
       </c>
       <c r="B135" s="10" t="inlineStr">
         <is>
-          <t>회의록</t>
+          <t>일정</t>
         </is>
       </c>
       <c r="C135" s="4" t="inlineStr">
         <is>
-          <t>회의록을 지우면 발표 내용도 함께 지워지는가?</t>
+          <t>구글·카카오 링크가 국내 «자동차» 길찾기를 여는가?</t>
         </is>
       </c>
       <c r="D135" s="4" t="inlineStr">
         <is>
-          <t>발표 내용이 있는 회의록을 지우고 남은 줄 확인</t>
+          <t>두 지도의 링크 형식을 각각 눌러 결과 확인</t>
         </is>
       </c>
       <c r="E135" s="11" t="inlineStr">
@@ -6547,12 +6547,12 @@
       <c r="G135" s="10" t="inlineStr"/>
       <c r="H135" s="4" t="inlineStr">
         <is>
-          <t>남으면 «회의록 본문의 일부» 로 이어 놓았는지 확인</t>
+          <t>열리면 그대로 쓰면 된다</t>
         </is>
       </c>
       <c r="I135" s="4" t="inlineStr">
         <is>
-          <t>1 → 0 · 안건은 «반대로» 남는다(기한·담당·Jira 가 걸려 있다)</t>
+          <t>🔴 열리지 않는다 — 구글은 국내 자동차 길찾기를 제공하지 않고, 카카오는 sName·eName 을 통째로 버린다(실측). 그래서 네이버 «화면»까지 열고 이름은 복사 단추로</t>
         </is>
       </c>
     </row>
@@ -6564,17 +6564,17 @@
       </c>
       <c r="B136" s="12" t="inlineStr">
         <is>
-          <t>회의록</t>
+          <t>일정</t>
         </is>
       </c>
       <c r="C136" s="13" t="inlineStr">
         <is>
-          <t>발표 내용도 낱말 찾기에 걸리는가?</t>
+          <t>이름 복사가 실패해도 «반드시» 알리는가?</t>
         </is>
       </c>
       <c r="D136" s="13" t="inlineStr">
         <is>
-          <t>본문에 없고 발표 내용에만 있는 낱말로 검색해 걸리는지 확인</t>
+          <t>clipboard 성공 · isSecureContext 를 꺼 http 흉내 · 두 길 모두 막음 셋으로 확인</t>
         </is>
       </c>
       <c r="E136" s="14" t="inlineStr">
@@ -6590,12 +6590,12 @@
       <c r="G136" s="12" t="inlineStr"/>
       <c r="H136" s="13" t="inlineStr">
         <is>
-          <t>안 나오면 검색이 훑는 칸에 들어갔는지 확인</t>
+          <t>아무 말이 없으면 promise 를 그대로 돌려주고 있는지 확인</t>
         </is>
       </c>
       <c r="I136" s="13" t="inlineStr">
         <is>
-          <t>「자재」(본문 없음·발표 있음)로 그 회의록 1건만 걸림</t>
+          <t>🔴 첫 판은 «복사도 안 되고 토스트도 안 떴다» · 고친 뒤 셋 다 토스트 확인</t>
         </is>
       </c>
     </row>
@@ -6607,17 +6607,17 @@
       </c>
       <c r="B137" s="10" t="inlineStr">
         <is>
-          <t>안건</t>
+          <t>휴가</t>
         </is>
       </c>
       <c r="C137" s="4" t="inlineStr">
         <is>
-          <t>안건에 보고자를 담당자와 «따로» 지정할 수 있는가?</t>
+          <t>지난 날짜에 넣으면 신청 메일이 «안» 가는가?</t>
         </is>
       </c>
       <c r="D137" s="4" t="inlineStr">
         <is>
-          <t>담당자·보고자를 다른 사람으로 등록한 뒤 보고자만 바꾸고 비워 본다</t>
+          <t>지난 날짜로 휴가를 넣고 서버 발송 기록 확인</t>
         </is>
       </c>
       <c r="E137" s="11" t="inlineStr">
@@ -6633,12 +6633,12 @@
       <c r="G137" s="10" t="inlineStr"/>
       <c r="H137" s="4" t="inlineStr">
         <is>
-          <t>한 칸만 남으면 마이그레이션 034 가 운영 DB 에 들어갔는지 확인</t>
+          <t>나가면 plan_date 와 오늘을 맞대는 판정 확인</t>
         </is>
       </c>
       <c r="I137" s="4" t="inlineStr">
         <is>
-          <t>담당 고광용 / 보고 이건호 → 윤기곤 → 비움. 담당자는 내내 그대로</t>
+          <t>로그 skip(backfill) — 9/07·9/05 넷(신청·취소) 다 안 감</t>
         </is>
       </c>
     </row>
@@ -6650,17 +6650,17 @@
       </c>
       <c r="B138" s="12" t="inlineStr">
         <is>
-          <t>배포</t>
+          <t>휴가</t>
         </is>
       </c>
       <c r="C138" s="13" t="inlineStr">
         <is>
-          <t>새 API 가 쓰는 DB 칸이 운영에 «먼저» 들어갔는가?</t>
+          <t>오늘·앞날은 «그대로» 신청 메일이 가는가?</t>
         </is>
       </c>
       <c r="D138" s="13" t="inlineStr">
         <is>
-          <t>배포 전 information_schema 로 칸·표 존재 확인</t>
+          <t>오늘·앞날로 넣고 서버 발송 기록 확인</t>
         </is>
       </c>
       <c r="E138" s="14" t="inlineStr">
@@ -6676,12 +6676,12 @@
       <c r="G138" s="12" t="inlineStr"/>
       <c r="H138" s="13" t="inlineStr">
         <is>
-          <t>없으면 배포를 멈추고 마이그레이션부터 넣는다</t>
+          <t>안 가면 판정이 지나치게 넓은지 확인</t>
         </is>
       </c>
       <c r="I138" s="13" t="inlineStr">
         <is>
-          <t>033~037 확인 후 배포 — 안 넣고 배포하면 새 API 가 500 으로 죽는다</t>
+          <t>9/10·9/13 신청·취소 넷 다 나감 — 막아 버리면 안 된다</t>
         </is>
       </c>
     </row>
@@ -6693,17 +6693,17 @@
       </c>
       <c r="B139" s="10" t="inlineStr">
         <is>
-          <t>배포</t>
+          <t>휴가</t>
         </is>
       </c>
       <c r="C139" s="4" t="inlineStr">
         <is>
-          <t>적어 둔 «적용 기록» 말고 DB 에 직접 물어 확인했는가?</t>
+          <t>지난 날짜가 «승인 대기»에 쌓이지 않는가?</t>
         </is>
       </c>
       <c r="D139" s="4" t="inlineStr">
         <is>
-          <t>CLAUDE.md 의 기록과 운영 DB 의 실제 칸을 대조</t>
+          <t>승인권자 계정으로 대기 목록을 넣기 전후로 세어 본다</t>
         </is>
       </c>
       <c r="E139" s="11" t="inlineStr">
@@ -6719,247 +6719,1564 @@
       <c r="G139" s="10" t="inlineStr"/>
       <c r="H139" s="4" t="inlineStr">
         <is>
+          <t>늘어나면 자동 승인이 안 걸린 것</t>
+        </is>
+      </c>
+      <c r="I139" s="4" t="inlineStr">
+        <is>
+          <t>넣기 전 0 → 지난 날짜 2건 넣은 뒤에도 0</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" s="12" t="inlineStr">
+        <is>
+          <t>TC-D-138</t>
+        </is>
+      </c>
+      <c r="B140" s="12" t="inlineStr">
+        <is>
+          <t>휴가</t>
+        </is>
+      </c>
+      <c r="C140" s="13" t="inlineStr">
+        <is>
+          <t>자동 승인된 것을 «사람이 승인한 것»과 구분할 수 있는가?</t>
+        </is>
+      </c>
+      <c r="D140" s="13" t="inlineStr">
+        <is>
+          <t>저장된 approval 과 approved_by_id 확인</t>
+        </is>
+      </c>
+      <c r="E140" s="14" t="inlineStr">
+        <is>
+          <t>적합</t>
+        </is>
+      </c>
+      <c r="F140" s="12" t="inlineStr">
+        <is>
+          <t>이건호</t>
+        </is>
+      </c>
+      <c r="G140" s="12" t="inlineStr"/>
+      <c r="H140" s="13" t="inlineStr">
+        <is>
+          <t>승인자가 채워지면 「누가 승인했다」가 거짓이 된다</t>
+        </is>
+      </c>
+      <c r="I140" s="13" t="inlineStr">
+        <is>
+          <t>approved + approved_by_id = null · 승인 시각은 찍힌다</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" s="10" t="inlineStr">
+        <is>
+          <t>TC-D-139</t>
+        </is>
+      </c>
+      <c r="B141" s="10" t="inlineStr">
+        <is>
+          <t>휴가</t>
+        </is>
+      </c>
+      <c r="C141" s="4" t="inlineStr">
+        <is>
+          <t>지난 날짜를 지울 때도 취소 메일이 «안» 가는가?</t>
+        </is>
+      </c>
+      <c r="D141" s="4" t="inlineStr">
+        <is>
+          <t>지난 날짜 건을 지우고 발송 기록 확인</t>
+        </is>
+      </c>
+      <c r="E141" s="11" t="inlineStr">
+        <is>
+          <t>적합</t>
+        </is>
+      </c>
+      <c r="F141" s="10" t="inlineStr">
+        <is>
+          <t>이건호</t>
+        </is>
+      </c>
+      <c r="G141" s="10" t="inlineStr"/>
+      <c r="H141" s="4" t="inlineStr">
+        <is>
+          <t>가면 취소 경로에도 같은 판정이 걸렸는지 확인</t>
+        </is>
+      </c>
+      <c r="I141" s="4" t="inlineStr">
+        <is>
+          <t>신청이 안 갔는데 취소만 가면 «없던 신청»이 취소된 것으로 읽힌다</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" s="12" t="inlineStr">
+        <is>
+          <t>TC-D-140</t>
+        </is>
+      </c>
+      <c r="B142" s="12" t="inlineStr">
+        <is>
+          <t>휴가</t>
+        </is>
+      </c>
+      <c r="C142" s="13" t="inlineStr">
+        <is>
+          <t>날짜가 섞였을 때 화면이 «갈라서» 묻는가?</t>
+        </is>
+      </c>
+      <c r="D142" s="13" t="inlineStr">
+        <is>
+          <t>지난 날짜와 오늘을 함께 골라 확인 창 문구를 읽는다</t>
+        </is>
+      </c>
+      <c r="E142" s="14" t="inlineStr">
+        <is>
+          <t>적합</t>
+        </is>
+      </c>
+      <c r="F142" s="12" t="inlineStr">
+        <is>
+          <t>이건호</t>
+        </is>
+      </c>
+      <c r="G142" s="12" t="inlineStr"/>
+      <c r="H142" s="13" t="inlineStr">
+        <is>
+          <t>한 줄로 뭉뚱그리면 어느 쪽이 갔는지 알 수 없다</t>
+        </is>
+      </c>
+      <c r="I142" s="13" t="inlineStr">
+        <is>
+          <t>「지난 1건은 정리 기록…나머지 1건만 신청 메일」 · 전부 지난 날짜면 「넣을까요?」</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" s="10" t="inlineStr">
+        <is>
+          <t>TC-D-141</t>
+        </is>
+      </c>
+      <c r="B143" s="10" t="inlineStr">
+        <is>
+          <t>휴가</t>
+        </is>
+      </c>
+      <c r="C143" s="4" t="inlineStr">
+        <is>
+          <t>시각을 고르면 시스템이 시간을 세는가?</t>
+        </is>
+      </c>
+      <c r="D143" s="4" t="inlineStr">
+        <is>
+          <t>종일·09:00~18:00·09:00~13:00 등 여덟 가지로 등록해 값 확인</t>
+        </is>
+      </c>
+      <c r="E143" s="11" t="inlineStr">
+        <is>
+          <t>적합</t>
+        </is>
+      </c>
+      <c r="F143" s="10" t="inlineStr">
+        <is>
+          <t>이건호</t>
+        </is>
+      </c>
+      <c r="G143" s="10" t="inlineStr"/>
+      <c r="H143" s="4" t="inlineStr">
+        <is>
+          <t>값이 다르면 근무·점심 시각 상수와 겹침 계산 확인</t>
+        </is>
+      </c>
+      <c r="I143" s="4" t="inlineStr">
+        <is>
+          <t>8/8 일치 — 종일 8 · 09~18 8 · 09~13 3 · 13~18 5 · 11~14 2 · 끝이 앞서면 0</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" s="12" t="inlineStr">
+        <is>
+          <t>TC-D-142</t>
+        </is>
+      </c>
+      <c r="B144" s="12" t="inlineStr">
+        <is>
+          <t>휴가</t>
+        </is>
+      </c>
+      <c r="C144" s="13" t="inlineStr">
+        <is>
+          <t>점심시간이 휴가에서 빠지는가?</t>
+        </is>
+      </c>
+      <c r="D144" s="13" t="inlineStr">
+        <is>
+          <t>09:00~13:00 으로 등록해 3시간인지 확인</t>
+        </is>
+      </c>
+      <c r="E144" s="14" t="inlineStr">
+        <is>
+          <t>적합</t>
+        </is>
+      </c>
+      <c r="F144" s="12" t="inlineStr">
+        <is>
+          <t>이건호</t>
+        </is>
+      </c>
+      <c r="G144" s="12" t="inlineStr"/>
+      <c r="H144" s="13" t="inlineStr">
+        <is>
+          <t>4시간이면 점심 구간과의 겹침을 빼는지 확인</t>
+        </is>
+      </c>
+      <c r="I144" s="13" t="inlineStr">
+        <is>
+          <t>3시간 — 점심 전까지(09~12)도 3시간이라 겹칠 때만 빠진다</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" s="10" t="inlineStr">
+        <is>
+          <t>TC-D-143</t>
+        </is>
+      </c>
+      <c r="B145" s="10" t="inlineStr">
+        <is>
+          <t>휴가</t>
+        </is>
+      </c>
+      <c r="C145" s="4" t="inlineStr">
+        <is>
+          <t>「반차」 단추가 사라지고 시각 고르개가 나오는가?</t>
+        </is>
+      </c>
+      <c r="D145" s="4" t="inlineStr">
+        <is>
+          <t>운영 화면에서 휴가 유형을 골라 단추 목록 확인</t>
+        </is>
+      </c>
+      <c r="E145" s="11" t="inlineStr">
+        <is>
+          <t>적합</t>
+        </is>
+      </c>
+      <c r="F145" s="10" t="inlineStr">
+        <is>
+          <t>이건호</t>
+        </is>
+      </c>
+      <c r="G145" s="10" t="inlineStr"/>
+      <c r="H145" s="4" t="inlineStr">
+        <is>
+          <t>반차가 남아 있으면 배포본이 옛것인지 확인</t>
+        </is>
+      </c>
+      <c r="I145" s="4" t="inlineStr">
+        <is>
+          <t>종류 연차·병가·포상·공가·기타 / 길이 종일(8시간)·시간 지정</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" s="12" t="inlineStr">
+        <is>
+          <t>TC-D-144</t>
+        </is>
+      </c>
+      <c r="B146" s="12" t="inlineStr">
+        <is>
+          <t>휴가</t>
+        </is>
+      </c>
+      <c r="C146" s="13" t="inlineStr">
+        <is>
+          <t>지난 휴가가 종일 8시간·반차 4시간으로 환산됐는가?</t>
+        </is>
+      </c>
+      <c r="D146" s="13" t="inlineStr">
+        <is>
+          <t>운영 DB 에 마이그레이션 035 적용 후 환산 결과 확인</t>
+        </is>
+      </c>
+      <c r="E146" s="14" t="inlineStr">
+        <is>
+          <t>적합</t>
+        </is>
+      </c>
+      <c r="F146" s="12" t="inlineStr">
+        <is>
+          <t>이건호</t>
+        </is>
+      </c>
+      <c r="G146" s="12" t="inlineStr"/>
+      <c r="H146" s="13" t="inlineStr">
+        <is>
+          <t>빈 값이 남으면 UPDATE 조건 확인</t>
+        </is>
+      </c>
+      <c r="I146" s="13" t="inlineStr">
+        <is>
+          <t>운영 5건 모두 종일 → 8시간 · 시간 없는 휴가 0건</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" s="10" t="inlineStr">
+        <is>
+          <t>TC-D-145</t>
+        </is>
+      </c>
+      <c r="B147" s="10" t="inlineStr">
+        <is>
+          <t>휴가</t>
+        </is>
+      </c>
+      <c r="C147" s="4" t="inlineStr">
+        <is>
+          <t>연차 집계가 «일과 시간» 을 함께 내는가?</t>
+        </is>
+      </c>
+      <c r="D147" s="4" t="inlineStr">
+        <is>
+          <t>연차 요약에서 부여·사용·잔여 값 확인</t>
+        </is>
+      </c>
+      <c r="E147" s="11" t="inlineStr">
+        <is>
+          <t>적합</t>
+        </is>
+      </c>
+      <c r="F147" s="10" t="inlineStr">
+        <is>
+          <t>이건호</t>
+        </is>
+      </c>
+      <c r="G147" s="10" t="inlineStr"/>
+      <c r="H147" s="4" t="inlineStr">
+        <is>
+          <t>한쪽만 나오면 집계 응답에 시간 칸이 있는지 확인</t>
+        </is>
+      </c>
+      <c r="I147" s="4" t="inlineStr">
+        <is>
+          <t>부여 21일/168시간 · 하루 8시간 · 잔여도 양쪽 표시</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" s="12" t="inlineStr">
+        <is>
+          <t>TC-D-146</t>
+        </is>
+      </c>
+      <c r="B148" s="12" t="inlineStr">
+        <is>
+          <t>휴가</t>
+        </is>
+      </c>
+      <c r="C148" s="13" t="inlineStr">
+        <is>
+          <t>「공가」를 종류로 고를 수 있고 사유를 적을 수 있는가?</t>
+        </is>
+      </c>
+      <c r="D148" s="13" t="inlineStr">
+        <is>
+          <t>운영 화면에서 공가를 고르고 사유 칸 확인</t>
+        </is>
+      </c>
+      <c r="E148" s="14" t="inlineStr">
+        <is>
+          <t>적합</t>
+        </is>
+      </c>
+      <c r="F148" s="12" t="inlineStr">
+        <is>
+          <t>이건호</t>
+        </is>
+      </c>
+      <c r="G148" s="12" t="inlineStr"/>
+      <c r="H148" s="13" t="inlineStr">
+        <is>
+          <t>안 보이면 마이그레이션 033 이 운영 DB 에 들어갔는지 확인</t>
+        </is>
+      </c>
+      <c r="I148" s="13" t="inlineStr">
+        <is>
+          <t>종류 다섯에 공가 확인(운영 화면) · 사유 칸은 같은 판 화면에서 확인 · 예비군·경조용</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" s="10" t="inlineStr">
+        <is>
+          <t>TC-D-147</t>
+        </is>
+      </c>
+      <c r="B149" s="10" t="inlineStr">
+        <is>
+          <t>회의록</t>
+        </is>
+      </c>
+      <c r="C149" s="4" t="inlineStr">
+        <is>
+          <t>작성자를 직원 목록에서 고르거나 직접 적을 수 있는가?</t>
+        </is>
+      </c>
+      <c r="D149" s="4" t="inlineStr">
+        <is>
+          <t>회의록을 만들며 두 가지 방식으로 저장한 뒤 다시 조회</t>
+        </is>
+      </c>
+      <c r="E149" s="11" t="inlineStr">
+        <is>
+          <t>적합</t>
+        </is>
+      </c>
+      <c r="F149" s="10" t="inlineStr">
+        <is>
+          <t>이건호</t>
+        </is>
+      </c>
+      <c r="G149" s="10" t="inlineStr"/>
+      <c r="H149" s="4" t="inlineStr">
+        <is>
+          <t>한쪽만 남으면 «둘 중 하나만» 담는 조건 확인</t>
+        </is>
+      </c>
+      <c r="I149" s="4" t="inlineStr">
+        <is>
+          <t>직접 입력 → 글자로 · 목록 선택 → 번호로. 양쪽에 동시에 남지 않는다</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" s="12" t="inlineStr">
+        <is>
+          <t>TC-D-148</t>
+        </is>
+      </c>
+      <c r="B150" s="12" t="inlineStr">
+        <is>
+          <t>회의록</t>
+        </is>
+      </c>
+      <c r="C150" s="13" t="inlineStr">
+        <is>
+          <t>회의 내용에 서식(굵게·크기·색)을 넣을 수 있는가?</t>
+        </is>
+      </c>
+      <c r="D150" s="13" t="inlineStr">
+        <is>
+          <t>글을 골라 B·크게·빨강을 눌러 실제 저장값 확인</t>
+        </is>
+      </c>
+      <c r="E150" s="14" t="inlineStr">
+        <is>
+          <t>적합</t>
+        </is>
+      </c>
+      <c r="F150" s="12" t="inlineStr">
+        <is>
+          <t>이건호</t>
+        </is>
+      </c>
+      <c r="G150" s="12" t="inlineStr"/>
+      <c r="H150" s="13" t="inlineStr">
+        <is>
+          <t>안 걸리면 고른 글이 풀렸는지(마우스 누름 차단) 확인</t>
+        </is>
+      </c>
+      <c r="I150" s="13" t="inlineStr">
+        <is>
+          <t>font-weight·font-size·color 가 걸리고 저장 후에도 남는다</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" s="10" t="inlineStr">
+        <is>
+          <t>TC-D-149</t>
+        </is>
+      </c>
+      <c r="B151" s="10" t="inlineStr">
+        <is>
+          <t>회의록</t>
+        </is>
+      </c>
+      <c r="C151" s="4" t="inlineStr">
+        <is>
+          <t>붙여 넣은 글이 «글자만» 들어오는가?</t>
+        </is>
+      </c>
+      <c r="D151" s="4" t="inlineStr">
+        <is>
+          <t>배경색·글꼴이 든 글을 편집기에 붙여 넣고 들어간 값 확인</t>
+        </is>
+      </c>
+      <c r="E151" s="11" t="inlineStr">
+        <is>
+          <t>적합</t>
+        </is>
+      </c>
+      <c r="F151" s="10" t="inlineStr">
+        <is>
+          <t>이건호</t>
+        </is>
+      </c>
+      <c r="G151" s="10" t="inlineStr"/>
+      <c r="H151" s="4" t="inlineStr">
+        <is>
+          <t>배경색이 따라오면 붙여 넣기 가로채기 확인</t>
+        </is>
+      </c>
+      <c r="I151" s="4" t="inlineStr">
+        <is>
+          <t>글자만 들어감 — background·font-family 안 따라옴 · 흰 바탕에 흰 글씨를 막는다</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" s="12" t="inlineStr">
+        <is>
+          <t>TC-D-150</t>
+        </is>
+      </c>
+      <c r="B152" s="12" t="inlineStr">
+        <is>
+          <t>회의록</t>
+        </is>
+      </c>
+      <c r="C152" s="13" t="inlineStr">
+        <is>
+          <t>옛 회의록(서식 없는 글)이 그대로 보이는가?</t>
+        </is>
+      </c>
+      <c r="D152" s="13" t="inlineStr">
+        <is>
+          <t>서식 없이 적힌 회의록을 열어 줄바꿈·본문 확인</t>
+        </is>
+      </c>
+      <c r="E152" s="14" t="inlineStr">
+        <is>
+          <t>적합</t>
+        </is>
+      </c>
+      <c r="F152" s="12" t="inlineStr">
+        <is>
+          <t>이건호</t>
+        </is>
+      </c>
+      <c r="G152" s="12" t="inlineStr"/>
+      <c r="H152" s="13" t="inlineStr">
+        <is>
+          <t>뭉개지면 글자를 서식으로 바꾸는 경로 확인</t>
+        </is>
+      </c>
+      <c r="I152" s="13" t="inlineStr">
+        <is>
+          <t>줄바꿈 유지 — 운영의 지난 주간회의로 확인</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" s="10" t="inlineStr">
+        <is>
+          <t>TC-D-151</t>
+        </is>
+      </c>
+      <c r="B153" s="10" t="inlineStr">
+        <is>
+          <t>회의록</t>
+        </is>
+      </c>
+      <c r="C153" s="4" t="inlineStr">
+        <is>
+          <t>위험한 글이 «보는 화면» 에서 걸러지는가?</t>
+        </is>
+      </c>
+      <c r="D153" s="4" t="inlineStr">
+        <is>
+          <t>DB 에 직접 심고 회의록을 열어 실행 여부 확인</t>
+        </is>
+      </c>
+      <c r="E153" s="11" t="inlineStr">
+        <is>
+          <t>적합</t>
+        </is>
+      </c>
+      <c r="F153" s="10" t="inlineStr">
+        <is>
+          <t>이건호</t>
+        </is>
+      </c>
+      <c r="G153" s="10" t="inlineStr"/>
+      <c r="H153" s="4" t="inlineStr">
+        <is>
+          <t>실행되면 그리기 직전의 거르개 확인</t>
+        </is>
+      </c>
+      <c r="I153" s="4" t="inlineStr">
+        <is>
+          <t>script·img·iframe 0개 · javascript: 주소 떨어짐 · 색·목록 서식은 남음</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" s="12" t="inlineStr">
+        <is>
+          <t>TC-D-152</t>
+        </is>
+      </c>
+      <c r="B154" s="12" t="inlineStr">
+        <is>
+          <t>회의록</t>
+        </is>
+      </c>
+      <c r="C154" s="13" t="inlineStr">
+        <is>
+          <t>위험한 글이 «고치는 화면» 에서도 걸러지는가?</t>
+        </is>
+      </c>
+      <c r="D154" s="13" t="inlineStr">
+        <is>
+          <t>같은 글로 [내용 수정] 을 눌러 실행 여부 확인</t>
+        </is>
+      </c>
+      <c r="E154" s="14" t="inlineStr">
+        <is>
+          <t>적합</t>
+        </is>
+      </c>
+      <c r="F154" s="12" t="inlineStr">
+        <is>
+          <t>이건호</t>
+        </is>
+      </c>
+      <c r="G154" s="12" t="inlineStr"/>
+      <c r="H154" s="13" t="inlineStr">
+        <is>
+          <t>실행되면 편집기에 담을 때도 거르는지 확인</t>
+        </is>
+      </c>
+      <c r="I154" s="13" t="inlineStr">
+        <is>
+          <t>🔴 처음 판은 여기서 &lt;img onerror&gt; 가 터졌다 — 고친 뒤 재확인</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" s="10" t="inlineStr">
+        <is>
+          <t>TC-D-153</t>
+        </is>
+      </c>
+      <c r="B155" s="10" t="inlineStr">
+        <is>
+          <t>회의록</t>
+        </is>
+      </c>
+      <c r="C155" s="4" t="inlineStr">
+        <is>
+          <t>발표 내용을 «본인 칸만» 고칠 수 있는가?</t>
+        </is>
+      </c>
+      <c r="D155" s="4" t="inlineStr">
+        <is>
+          <t>다른 사람 번호로 저장 요청</t>
+        </is>
+      </c>
+      <c r="E155" s="11" t="inlineStr">
+        <is>
+          <t>적합</t>
+        </is>
+      </c>
+      <c r="F155" s="10" t="inlineStr">
+        <is>
+          <t>이건호</t>
+        </is>
+      </c>
+      <c r="G155" s="10" t="inlineStr"/>
+      <c r="H155" s="4" t="inlineStr">
+        <is>
+          <t>저장되면 주소의 번호와 세션을 맞대는지 확인</t>
+        </is>
+      </c>
+      <c r="I155" s="4" t="inlineStr">
+        <is>
+          <t>403 「본인의 발표 내용만 적을 수 있습니다」</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" s="12" t="inlineStr">
+        <is>
+          <t>TC-D-154</t>
+        </is>
+      </c>
+      <c r="B156" s="12" t="inlineStr">
+        <is>
+          <t>회의록</t>
+        </is>
+      </c>
+      <c r="C156" s="13" t="inlineStr">
+        <is>
+          <t>관리자는 남의 발표 내용을 대신 넣을 수 있는가?</t>
+        </is>
+      </c>
+      <c r="D156" s="13" t="inlineStr">
+        <is>
+          <t>관리자 계정으로 다른 사람 칸에 저장</t>
+        </is>
+      </c>
+      <c r="E156" s="14" t="inlineStr">
+        <is>
+          <t>적합</t>
+        </is>
+      </c>
+      <c r="F156" s="12" t="inlineStr">
+        <is>
+          <t>이건호</t>
+        </is>
+      </c>
+      <c r="G156" s="12" t="inlineStr"/>
+      <c r="H156" s="13" t="inlineStr">
+        <is>
+          <t>막히면 등급 판정 확인</t>
+        </is>
+      </c>
+      <c r="I156" s="13" t="inlineStr">
+        <is>
+          <t>200 — 대리 입력은 허용한다</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" s="10" t="inlineStr">
+        <is>
+          <t>TC-D-155</t>
+        </is>
+      </c>
+      <c r="B157" s="10" t="inlineStr">
+        <is>
+          <t>회의록</t>
+        </is>
+      </c>
+      <c r="C157" s="4" t="inlineStr">
+        <is>
+          <t>한 사람이 프로젝트마다 나눠 적을 수 있는가?</t>
+        </is>
+      </c>
+      <c r="D157" s="4" t="inlineStr">
+        <is>
+          <t>같은 사람으로 프로젝트 둘 + 미지정 하나를 저장해 줄 수 확인</t>
+        </is>
+      </c>
+      <c r="E157" s="11" t="inlineStr">
+        <is>
+          <t>적합</t>
+        </is>
+      </c>
+      <c r="F157" s="10" t="inlineStr">
+        <is>
+          <t>이건호</t>
+        </is>
+      </c>
+      <c r="G157" s="10" t="inlineStr"/>
+      <c r="H157" s="4" t="inlineStr">
+        <is>
+          <t>한 줄로 덮이면 열쇠에 프로젝트가 들어갔는지 확인</t>
+        </is>
+      </c>
+      <c r="I157" s="4" t="inlineStr">
+        <is>
+          <t>3줄 유지 — 열쇠는 «회의 × 사람 × 프로젝트»</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" s="12" t="inlineStr">
+        <is>
+          <t>TC-D-156</t>
+        </is>
+      </c>
+      <c r="B158" s="12" t="inlineStr">
+        <is>
+          <t>회의록</t>
+        </is>
+      </c>
+      <c r="C158" s="13" t="inlineStr">
+        <is>
+          <t>같은 사람·같은 프로젝트에 다시 적으면 덮어쓰는가?</t>
+        </is>
+      </c>
+      <c r="D158" s="13" t="inlineStr">
+        <is>
+          <t>같은 자리에 두 번 저장해 줄 수와 내용 확인</t>
+        </is>
+      </c>
+      <c r="E158" s="14" t="inlineStr">
+        <is>
+          <t>적합</t>
+        </is>
+      </c>
+      <c r="F158" s="12" t="inlineStr">
+        <is>
+          <t>이건호</t>
+        </is>
+      </c>
+      <c r="G158" s="12" t="inlineStr"/>
+      <c r="H158" s="13" t="inlineStr">
+        <is>
+          <t>줄이 늘면 겹침 열쇠 확인</t>
+        </is>
+      </c>
+      <c r="I158" s="13" t="inlineStr">
+        <is>
+          <t>줄 수 그대로 · 내용만 바뀜</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" s="10" t="inlineStr">
+        <is>
+          <t>TC-D-157</t>
+        </is>
+      </c>
+      <c r="B159" s="10" t="inlineStr">
+        <is>
+          <t>회의록</t>
+        </is>
+      </c>
+      <c r="C159" s="4" t="inlineStr">
+        <is>
+          <t>프로젝트를 안 고른 줄이 여러 개로 쌓이지 않는가?</t>
+        </is>
+      </c>
+      <c r="D159" s="4" t="inlineStr">
+        <is>
+          <t>프로젝트 없이 두 번 저장해 줄 수 확인</t>
+        </is>
+      </c>
+      <c r="E159" s="11" t="inlineStr">
+        <is>
+          <t>적합</t>
+        </is>
+      </c>
+      <c r="F159" s="10" t="inlineStr">
+        <is>
+          <t>이건호</t>
+        </is>
+      </c>
+      <c r="G159" s="10" t="inlineStr"/>
+      <c r="H159" s="4" t="inlineStr">
+        <is>
+          <t>두 줄이면 NULL 을 빈 글자로 바꿔 잠갔는지 확인</t>
+        </is>
+      </c>
+      <c r="I159" s="4" t="inlineStr">
+        <is>
+          <t>🔴 NULL 끼리는 서로 같지 않아 그냥 UNIQUE 로는 «안 막힌다» · 1줄 확인</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" s="12" t="inlineStr">
+        <is>
+          <t>TC-D-158</t>
+        </is>
+      </c>
+      <c r="B160" s="12" t="inlineStr">
+        <is>
+          <t>회의록</t>
+        </is>
+      </c>
+      <c r="C160" s="13" t="inlineStr">
+        <is>
+          <t>프로젝트를 옮기면 옛 줄이 남지 않는가?</t>
+        </is>
+      </c>
+      <c r="D160" s="13" t="inlineStr">
+        <is>
+          <t>적어 둔 줄의 프로젝트를 바꿔 저장한 뒤 목록 확인</t>
+        </is>
+      </c>
+      <c r="E160" s="14" t="inlineStr">
+        <is>
+          <t>적합</t>
+        </is>
+      </c>
+      <c r="F160" s="12" t="inlineStr">
+        <is>
+          <t>이건호</t>
+        </is>
+      </c>
+      <c r="G160" s="12" t="inlineStr"/>
+      <c r="H160" s="13" t="inlineStr">
+        <is>
+          <t>두 자리에 남으면 옮길 때 옛 줄을 먼저 지우는지 확인</t>
+        </is>
+      </c>
+      <c r="I160" s="13" t="inlineStr">
+        <is>
+          <t>화면에서 확인 — 개수 3 그대로, 옛 프로젝트에서 사라짐</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" s="10" t="inlineStr">
+        <is>
+          <t>TC-D-159</t>
+        </is>
+      </c>
+      <c r="B161" s="10" t="inlineStr">
+        <is>
+          <t>회의록</t>
+        </is>
+      </c>
+      <c r="C161" s="4" t="inlineStr">
+        <is>
+          <t>적어 둔 것이 본문 아래에 «한 박스» 로 이어 붙는가?</t>
+        </is>
+      </c>
+      <c r="D161" s="4" t="inlineStr">
+        <is>
+          <t>회의록을 열어 본문과 발표 내용이 한 상자에 나오는지 확인</t>
+        </is>
+      </c>
+      <c r="E161" s="11" t="inlineStr">
+        <is>
+          <t>적합</t>
+        </is>
+      </c>
+      <c r="F161" s="10" t="inlineStr">
+        <is>
+          <t>이건호</t>
+        </is>
+      </c>
+      <c r="G161" s="10" t="inlineStr"/>
+      <c r="H161" s="4" t="inlineStr">
+        <is>
+          <t>따로 나오면 이어 붙이는 자리 확인</t>
+        </is>
+      </c>
+      <c r="I161" s="4" t="inlineStr">
+        <is>
+          <t>🗣 이름과 📁 프로젝트가 함께 붙는다</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" s="12" t="inlineStr">
+        <is>
+          <t>TC-D-160</t>
+        </is>
+      </c>
+      <c r="B162" s="12" t="inlineStr">
+        <is>
+          <t>회의록</t>
+        </is>
+      </c>
+      <c r="C162" s="13" t="inlineStr">
+        <is>
+          <t>같은 글을 인원별·프로젝트별 두 가지로 묶어 볼 수 있는가?</t>
+        </is>
+      </c>
+      <c r="D162" s="13" t="inlineStr">
+        <is>
+          <t>[🗣 인원별]/[📁 프로젝트별] 을 눌러 묶음이 뒤집히는지 확인</t>
+        </is>
+      </c>
+      <c r="E162" s="14" t="inlineStr">
+        <is>
+          <t>적합</t>
+        </is>
+      </c>
+      <c r="F162" s="12" t="inlineStr">
+        <is>
+          <t>이건호</t>
+        </is>
+      </c>
+      <c r="G162" s="12" t="inlineStr"/>
+      <c r="H162" s="13" t="inlineStr">
+        <is>
+          <t>한쪽만 되면 묶는 기준만 바꾸는지 확인</t>
+        </is>
+      </c>
+      <c r="I162" s="13" t="inlineStr">
+        <is>
+          <t>인원별=사람→프로젝트 · 프로젝트별=프로젝트→사람 · 미지정은 늘 맨 뒤</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" s="10" t="inlineStr">
+        <is>
+          <t>TC-D-161</t>
+        </is>
+      </c>
+      <c r="B163" s="10" t="inlineStr">
+        <is>
+          <t>회의록</t>
+        </is>
+      </c>
+      <c r="C163" s="4" t="inlineStr">
+        <is>
+          <t>회의록을 지우면 발표 내용도 함께 지워지는가?</t>
+        </is>
+      </c>
+      <c r="D163" s="4" t="inlineStr">
+        <is>
+          <t>발표 내용이 있는 회의록을 지우고 남은 줄 확인</t>
+        </is>
+      </c>
+      <c r="E163" s="11" t="inlineStr">
+        <is>
+          <t>적합</t>
+        </is>
+      </c>
+      <c r="F163" s="10" t="inlineStr">
+        <is>
+          <t>이건호</t>
+        </is>
+      </c>
+      <c r="G163" s="10" t="inlineStr"/>
+      <c r="H163" s="4" t="inlineStr">
+        <is>
+          <t>남으면 «회의록 본문의 일부» 로 이어 놓았는지 확인</t>
+        </is>
+      </c>
+      <c r="I163" s="4" t="inlineStr">
+        <is>
+          <t>1 → 0 · 안건은 «반대로» 남는다(기한·담당·Jira 가 걸려 있다)</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" s="12" t="inlineStr">
+        <is>
+          <t>TC-D-162</t>
+        </is>
+      </c>
+      <c r="B164" s="12" t="inlineStr">
+        <is>
+          <t>회의록</t>
+        </is>
+      </c>
+      <c r="C164" s="13" t="inlineStr">
+        <is>
+          <t>발표 내용도 낱말 찾기에 걸리는가?</t>
+        </is>
+      </c>
+      <c r="D164" s="13" t="inlineStr">
+        <is>
+          <t>본문에 없고 발표 내용에만 있는 낱말로 검색해 걸리는지 확인</t>
+        </is>
+      </c>
+      <c r="E164" s="14" t="inlineStr">
+        <is>
+          <t>적합</t>
+        </is>
+      </c>
+      <c r="F164" s="12" t="inlineStr">
+        <is>
+          <t>이건호</t>
+        </is>
+      </c>
+      <c r="G164" s="12" t="inlineStr"/>
+      <c r="H164" s="13" t="inlineStr">
+        <is>
+          <t>안 나오면 검색이 훑는 칸에 들어갔는지 확인</t>
+        </is>
+      </c>
+      <c r="I164" s="13" t="inlineStr">
+        <is>
+          <t>「자재」(본문 없음·발표 있음)로 그 회의록 1건만 걸림</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" s="10" t="inlineStr">
+        <is>
+          <t>TC-D-163</t>
+        </is>
+      </c>
+      <c r="B165" s="10" t="inlineStr">
+        <is>
+          <t>안건</t>
+        </is>
+      </c>
+      <c r="C165" s="4" t="inlineStr">
+        <is>
+          <t>안건에 보고자를 담당자와 «따로» 지정할 수 있는가?</t>
+        </is>
+      </c>
+      <c r="D165" s="4" t="inlineStr">
+        <is>
+          <t>담당자·보고자를 다른 사람으로 등록한 뒤 보고자만 바꾸고 비워 본다</t>
+        </is>
+      </c>
+      <c r="E165" s="11" t="inlineStr">
+        <is>
+          <t>적합</t>
+        </is>
+      </c>
+      <c r="F165" s="10" t="inlineStr">
+        <is>
+          <t>이건호</t>
+        </is>
+      </c>
+      <c r="G165" s="10" t="inlineStr"/>
+      <c r="H165" s="4" t="inlineStr">
+        <is>
+          <t>한 칸만 남으면 마이그레이션 034 가 운영 DB 에 들어갔는지 확인</t>
+        </is>
+      </c>
+      <c r="I165" s="4" t="inlineStr">
+        <is>
+          <t>담당 고광용 / 보고 이건호 → 윤기곤 → 비움. 담당자는 내내 그대로</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" s="12" t="inlineStr">
+        <is>
+          <t>TC-D-164</t>
+        </is>
+      </c>
+      <c r="B166" s="12" t="inlineStr">
+        <is>
+          <t>배포</t>
+        </is>
+      </c>
+      <c r="C166" s="13" t="inlineStr">
+        <is>
+          <t>새 API 가 쓰는 DB 칸이 운영에 «먼저» 들어갔는가?</t>
+        </is>
+      </c>
+      <c r="D166" s="13" t="inlineStr">
+        <is>
+          <t>배포 전 information_schema 로 칸·표 존재 확인</t>
+        </is>
+      </c>
+      <c r="E166" s="14" t="inlineStr">
+        <is>
+          <t>적합</t>
+        </is>
+      </c>
+      <c r="F166" s="12" t="inlineStr">
+        <is>
+          <t>이건호</t>
+        </is>
+      </c>
+      <c r="G166" s="12" t="inlineStr"/>
+      <c r="H166" s="13" t="inlineStr">
+        <is>
+          <t>없으면 배포를 멈추고 마이그레이션부터 넣는다</t>
+        </is>
+      </c>
+      <c r="I166" s="13" t="inlineStr">
+        <is>
+          <t>033~037 확인 후 배포 — 안 넣고 배포하면 새 API 가 500 으로 죽는다</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" s="10" t="inlineStr">
+        <is>
+          <t>TC-D-165</t>
+        </is>
+      </c>
+      <c r="B167" s="10" t="inlineStr">
+        <is>
+          <t>배포</t>
+        </is>
+      </c>
+      <c r="C167" s="4" t="inlineStr">
+        <is>
+          <t>적어 둔 «적용 기록» 말고 DB 에 직접 물어 확인했는가?</t>
+        </is>
+      </c>
+      <c r="D167" s="4" t="inlineStr">
+        <is>
+          <t>CLAUDE.md 의 기록과 운영 DB 의 실제 칸을 대조</t>
+        </is>
+      </c>
+      <c r="E167" s="11" t="inlineStr">
+        <is>
+          <t>적합</t>
+        </is>
+      </c>
+      <c r="F167" s="10" t="inlineStr">
+        <is>
+          <t>이건호</t>
+        </is>
+      </c>
+      <c r="G167" s="10" t="inlineStr"/>
+      <c r="H167" s="4" t="inlineStr">
+        <is>
           <t>다르면 DB 를 믿고 기록을 고친다</t>
         </is>
       </c>
-      <c r="I139" s="4" t="inlineStr">
+      <c r="I167" s="4" t="inlineStr">
         <is>
           <t>🔴 031·032 는 「테스트에만」 이라 적혀 있었으나 운영에 이미 들어가 있었다</t>
         </is>
       </c>
     </row>
-    <row r="140" ht="20" customHeight="1">
-      <c r="A140" s="9" t="inlineStr">
+    <row r="168" ht="20" customHeight="1">
+      <c r="A168" s="9" t="inlineStr">
         <is>
           <t>■ 미수행 — 자원·현장 조건이 갖춰져야 할 수 있다. 함께 실어 「전부 확인했다」로 읽히지 않게 한다.</t>
         </is>
       </c>
     </row>
-    <row r="141">
-      <c r="A141" s="15" t="inlineStr">
+    <row r="169">
+      <c r="A169" s="15" t="inlineStr">
         <is>
           <t>TC-DP-01</t>
         </is>
       </c>
-      <c r="B141" s="15" t="inlineStr">
+      <c r="B169" s="15" t="inlineStr">
         <is>
           <t>정산</t>
         </is>
       </c>
-      <c r="C141" s="16" t="inlineStr">
+      <c r="C169" s="16" t="inlineStr">
         <is>
           <t>한 달을 실제로 정산해 입금·환급까지 마칠 수 있는가?</t>
         </is>
       </c>
-      <c r="D141" s="16" t="inlineStr">
+      <c r="D169" s="16" t="inlineStr">
         <is>
           <t>한 달 운영 후 실제 정산 1회전 수행</t>
         </is>
       </c>
-      <c r="E141" s="17" t="inlineStr">
+      <c r="E169" s="17" t="inlineStr">
         <is>
           <t>미수행</t>
         </is>
       </c>
-      <c r="F141" s="15" t="inlineStr"/>
-      <c r="G141" s="15" t="inlineStr"/>
-      <c r="H141" s="16" t="inlineStr">
+      <c r="F169" s="15" t="inlineStr"/>
+      <c r="G169" s="15" t="inlineStr"/>
+      <c r="H169" s="16" t="inlineStr">
         <is>
           <t>운영 데이터가 쌓여야 한다 — 사용자가 직접 해 보고 알려 주기로 함(2026-08-24)</t>
         </is>
       </c>
-      <c r="I141" s="16" t="inlineStr"/>
-    </row>
-    <row r="142">
-      <c r="A142" s="15" t="inlineStr">
+      <c r="I169" s="16" t="inlineStr"/>
+    </row>
+    <row r="170">
+      <c r="A170" s="15" t="inlineStr">
         <is>
           <t>TC-DP-02</t>
         </is>
       </c>
-      <c r="B142" s="15" t="inlineStr">
+      <c r="B170" s="15" t="inlineStr">
         <is>
           <t>메일</t>
         </is>
       </c>
-      <c r="C142" s="16" t="inlineStr">
+      <c r="C170" s="16" t="inlineStr">
         <is>
           <t>각자 실제 앱 비밀번호로 등록해 본인 주소에서 메일이 나가는가?</t>
         </is>
       </c>
-      <c r="D142" s="16" t="inlineStr">
+      <c r="D170" s="16" t="inlineStr">
         <is>
           <t>직원 7명이 각자 다음 메일에서 앱 비밀번호를 발급받아 등록</t>
         </is>
       </c>
-      <c r="E142" s="17" t="inlineStr">
+      <c r="E170" s="17" t="inlineStr">
         <is>
           <t>미수행</t>
         </is>
       </c>
-      <c r="F142" s="15" t="inlineStr"/>
-      <c r="G142" s="15" t="inlineStr"/>
-      <c r="H142" s="16" t="inlineStr"/>
-      <c r="I142" s="16" t="inlineStr">
+      <c r="F170" s="15" t="inlineStr"/>
+      <c r="G170" s="15" t="inlineStr"/>
+      <c r="H170" s="16" t="inlineStr"/>
+      <c r="I170" s="16" t="inlineStr">
         <is>
           <t>비밀번호는 본인만 다룰 수 있어 대신 확인할 수 없다</t>
         </is>
       </c>
     </row>
-    <row r="143">
-      <c r="A143" s="15" t="inlineStr">
+    <row r="171">
+      <c r="A171" s="15" t="inlineStr">
         <is>
           <t>TC-DP-03</t>
         </is>
       </c>
-      <c r="B143" s="15" t="inlineStr">
+      <c r="B171" s="15" t="inlineStr">
         <is>
           <t>휴가</t>
         </is>
       </c>
-      <c r="C143" s="16" t="inlineStr">
+      <c r="C171" s="16" t="inlineStr">
         <is>
           <t>실제 휴가를 신청·승인해 양쪽 메일이 도착하는가?</t>
         </is>
       </c>
-      <c r="D143" s="16" t="inlineStr">
+      <c r="D171" s="16" t="inlineStr">
         <is>
           <t>직원이 신청하고 대표이사가 승인 — 두 통 모두 수신 확인</t>
         </is>
       </c>
-      <c r="E143" s="17" t="inlineStr">
+      <c r="E171" s="17" t="inlineStr">
         <is>
           <t>미수행</t>
         </is>
       </c>
-      <c r="F143" s="15" t="inlineStr"/>
-      <c r="G143" s="15" t="inlineStr"/>
-      <c r="H143" s="16" t="inlineStr"/>
-      <c r="I143" s="16" t="inlineStr">
+      <c r="F171" s="15" t="inlineStr"/>
+      <c r="G171" s="15" t="inlineStr"/>
+      <c r="H171" s="16" t="inlineStr"/>
+      <c r="I171" s="16" t="inlineStr">
         <is>
           <t>승인 권한자가 직접 해야 한다</t>
         </is>
       </c>
     </row>
-    <row r="144">
-      <c r="A144" s="15" t="inlineStr">
+    <row r="172">
+      <c r="A172" s="15" t="inlineStr">
         <is>
           <t>TC-DP-04</t>
         </is>
       </c>
-      <c r="B144" s="15" t="inlineStr">
+      <c r="B172" s="15" t="inlineStr">
         <is>
           <t>휴가</t>
         </is>
       </c>
-      <c r="C144" s="16" t="inlineStr">
+      <c r="C172" s="16" t="inlineStr">
         <is>
           <t>공가를 쓰면 연차 잔여가 그대로인가?</t>
         </is>
       </c>
-      <c r="D144" s="16" t="inlineStr">
+      <c r="D172" s="16" t="inlineStr">
         <is>
           <t>공가를 실제로 등록한 뒤 연차 요약의 사용·잔여 확인</t>
         </is>
       </c>
-      <c r="E144" s="17" t="inlineStr">
+      <c r="E172" s="17" t="inlineStr">
         <is>
           <t>미수행</t>
         </is>
       </c>
-      <c r="F144" s="15" t="inlineStr"/>
-      <c r="G144" s="15" t="inlineStr"/>
-      <c r="H144" s="16" t="inlineStr">
+      <c r="F172" s="15" t="inlineStr"/>
+      <c r="G172" s="15" t="inlineStr"/>
+      <c r="H172" s="16" t="inlineStr">
         <is>
           <t>운영에 공가 기록이 아직 없다 — 처음 쓰실 때 함께 확인</t>
         </is>
       </c>
-      <c r="I144" s="16" t="inlineStr"/>
-    </row>
-    <row r="145">
-      <c r="A145" s="15" t="inlineStr">
+      <c r="I172" s="16" t="inlineStr"/>
+    </row>
+    <row r="173">
+      <c r="A173" s="15" t="inlineStr">
         <is>
           <t>TC-DP-05</t>
         </is>
       </c>
-      <c r="B145" s="15" t="inlineStr">
+      <c r="B173" s="15" t="inlineStr">
         <is>
           <t>안건</t>
         </is>
       </c>
-      <c r="C145" s="16" t="inlineStr">
+      <c r="C173" s="16" t="inlineStr">
         <is>
           <t>Jira 로 올릴 때 제목 뒤에 «_보고자» 가 붙는가?</t>
         </is>
       </c>
-      <c r="D145" s="16" t="inlineStr">
+      <c r="D173" s="16" t="inlineStr">
         <is>
           <t>보고자를 넣은 안건을 Jira 로 올려 제목 확인</t>
         </is>
       </c>
-      <c r="E145" s="17" t="inlineStr">
+      <c r="E173" s="17" t="inlineStr">
         <is>
           <t>미수행</t>
         </is>
       </c>
-      <c r="F145" s="15" t="inlineStr"/>
-      <c r="G145" s="15" t="inlineStr"/>
-      <c r="H145" s="16" t="inlineStr">
+      <c r="F173" s="15" t="inlineStr"/>
+      <c r="G173" s="15" t="inlineStr"/>
+      <c r="H173" s="16" t="inlineStr">
         <is>
           <t>실제 Jira 이슈가 만들어지므로 시험용으로 올리지 않았다</t>
         </is>
       </c>
-      <c r="I145" s="16" t="inlineStr">
+      <c r="I173" s="16" t="inlineStr">
         <is>
           <t>여러 번 올려도 겹쳐 붙지 않아야 한다</t>
         </is>
       </c>
     </row>
-    <row r="146">
-      <c r="A146" s="15" t="inlineStr">
+    <row r="174">
+      <c r="A174" s="15" t="inlineStr">
         <is>
           <t>TC-DP-06</t>
         </is>
       </c>
-      <c r="B146" s="15" t="inlineStr">
+      <c r="B174" s="15" t="inlineStr">
         <is>
           <t>회의록</t>
         </is>
       </c>
-      <c r="C146" s="16" t="inlineStr">
+      <c r="C174" s="16" t="inlineStr">
         <is>
           <t>여러 사람이 «동시에» 자기 칸을 적어도 부딪히지 않는가?</t>
         </is>
       </c>
-      <c r="D146" s="16" t="inlineStr">
+      <c r="D174" s="16" t="inlineStr">
         <is>
           <t>두 사람이 같은 회의록을 동시에 열고 각자 저장</t>
         </is>
       </c>
-      <c r="E146" s="17" t="inlineStr">
+      <c r="E174" s="17" t="inlineStr">
         <is>
           <t>미수행</t>
         </is>
       </c>
-      <c r="F146" s="15" t="inlineStr"/>
-      <c r="G146" s="15" t="inlineStr"/>
-      <c r="H146" s="16" t="inlineStr">
+      <c r="F174" s="15" t="inlineStr"/>
+      <c r="G174" s="15" t="inlineStr"/>
+      <c r="H174" s="16" t="inlineStr">
         <is>
           <t>사람이 둘 이상 있어야 한다 — 실제 회의에서 확인</t>
         </is>
       </c>
-      <c r="I146" s="16" t="inlineStr">
+      <c r="I174" s="16" t="inlineStr">
         <is>
           <t>칸을 나눈 것이 이 문제를 없애기 위한 설계다</t>
+        </is>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" s="15" t="inlineStr">
+        <is>
+          <t>TC-DP-07</t>
+        </is>
+      </c>
+      <c r="B175" s="15" t="inlineStr">
+        <is>
+          <t>하이패스</t>
+        </is>
+      </c>
+      <c r="C175" s="16" t="inlineStr">
+        <is>
+          <t>실적 창의 하이패스 «고르기 화면» 이 제대로 뜨는가?</t>
+        </is>
+      </c>
+      <c r="D175" s="16" t="inlineStr">
+        <is>
+          <t>실적 창을 열어 그날 통행 목록·체크·합계 잠금 확인</t>
+        </is>
+      </c>
+      <c r="E175" s="17" t="inlineStr">
+        <is>
+          <t>미수행</t>
+        </is>
+      </c>
+      <c r="F175" s="15" t="inlineStr"/>
+      <c r="G175" s="15" t="inlineStr"/>
+      <c r="H175" s="16" t="inlineStr">
+        <is>
+          <t>브라우저 패널이 스케줄 화면에서 반복해 멎어 눈으로 확인하지 못했다</t>
+        </is>
+      </c>
+      <c r="I175" s="16" t="inlineStr">
+        <is>
+          <t>서버·API 쪽은 확인했다(TC-D 하이패스 항목). 배포본에서 눌러 확인할 것</t>
+        </is>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" s="15" t="inlineStr">
+        <is>
+          <t>TC-DP-08</t>
+        </is>
+      </c>
+      <c r="B176" s="15" t="inlineStr">
+        <is>
+          <t>하이패스</t>
+        </is>
+      </c>
+      <c r="C176" s="16" t="inlineStr">
+        <is>
+          <t>건별 하이패스 메일이 직원에게 도착하는가?</t>
+        </is>
+      </c>
+      <c r="D176" s="16" t="inlineStr">
+        <is>
+          <t>「메일 보내기」를 눌러 실제 수신 확인</t>
+        </is>
+      </c>
+      <c r="E176" s="17" t="inlineStr">
+        <is>
+          <t>미수행</t>
+        </is>
+      </c>
+      <c r="F176" s="15" t="inlineStr"/>
+      <c r="G176" s="15" t="inlineStr"/>
+      <c r="H176" s="16" t="inlineStr">
+        <is>
+          <t>실제 직원에게 나가므로 승인 전까지 누르지 않았다</t>
+        </is>
+      </c>
+      <c r="I176" s="16" t="inlineStr"/>
+    </row>
+    <row r="177">
+      <c r="A177" s="15" t="inlineStr">
+        <is>
+          <t>TC-DP-09</t>
+        </is>
+      </c>
+      <c r="B177" s="15" t="inlineStr">
+        <is>
+          <t>일정</t>
+        </is>
+      </c>
+      <c r="C177" s="16" t="inlineStr">
+        <is>
+          <t>네이버 길찾기 링크가 실제로 열리는가?</t>
+        </is>
+      </c>
+      <c r="D177" s="16" t="inlineStr">
+        <is>
+          <t>「이동」 일정에서 링크를 눌러 길찾기 화면 확인</t>
+        </is>
+      </c>
+      <c r="E177" s="17" t="inlineStr">
+        <is>
+          <t>미수행</t>
+        </is>
+      </c>
+      <c r="F177" s="15" t="inlineStr"/>
+      <c r="G177" s="15" t="inlineStr"/>
+      <c r="H177" s="16" t="inlineStr">
+        <is>
+          <t>브라우저 패널이 map.naver.com 을 정책으로 막는다</t>
+        </is>
+      </c>
+      <c r="I177" s="16" t="inlineStr">
+        <is>
+          <t>배포본에서 눌러 확인할 것</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="2">
+    <mergeCell ref="A168:I168"/>
     <mergeCell ref="A2:I2"/>
-    <mergeCell ref="A140:I140"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation sqref="E2:E146" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="E2:E177" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"적합,부적합,미수행"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>